<commit_message>
Add Marks 2026 JAMA NetOpen literature note + outreach tracker update
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outreach/outreach_tracker.xlsx
+++ b/outreach/outreach_tracker.xlsx
@@ -71,7 +71,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -90,6 +90,13 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="00FFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00D9D9D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -455,7 +462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J6"/>
+  <dimension ref="A1:J7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -758,6 +765,50 @@
         </is>
       </c>
     </row>
+    <row r="7" ht="60" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Ethan Goh, MD, MS</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Stanford (ARISE / HAILS)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ethangoh@stanford.edu</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Goh 2024 — RCT LLM vs clinicians (JAMA Netw Open); Goh 2025 Nature Med (mgmt reasoning)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Peer / evaluation methodology (not data)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Held</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Email drafted; sending paused pending new MIMIC hidden-dx benchmark results</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Stanford ARISE Exec Director; Assoc Editor BMJ Digital Health &amp; AI; independent of UCSF/Boston/Houston clusters</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="G2:G1000">
     <cfRule type="cellIs" priority="1" operator="equal" dxfId="0">
@@ -769,6 +820,9 @@
     <cfRule type="cellIs" priority="3" operator="equal" dxfId="2">
       <formula>"No"</formula>
     </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" dxfId="3">
+      <formula>"Held"</formula>
+    </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>